<commit_message>
Agregar nombres de matrices al excel dummies
</commit_message>
<xml_diff>
--- a/Prueba_Reconstruccion_MIP_Dummies.xlsx
+++ b/Prueba_Reconstruccion_MIP_Dummies.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0_Leer_primero" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_Mapa_simple" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Una_celda_Z" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Cierre_sin_susto" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_De_Z_a_A_L" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Simulador_facil" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_Glosario" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0_Nombres_matrices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_Mapa_simple" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Una_celda_Z" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Cierre_sin_susto" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_De_Z_a_A_L" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Simulador_facil" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_Glosario" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -657,7 +658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -730,34 +731,46 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>La celda ejemplo</t>
+          <t>Los nombres</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Calculamos cuanto le vende 'Alimentos e Bebidas' a 'Comércio'.</t>
+          <t>La hoja 0_Nombres_matrices lista el nombre de cada matriz, su simbolo y para que sirve.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>El cierre</t>
+          <t>La celda ejemplo</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Si queda una demanda final negativa muy pequena, la conciliamos con regla trazable; si es material, se deja alerta.</t>
+          <t>Calculamos cuanto le vende 'Alimentos e Bebidas' a 'Comércio'.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
+          <t>El cierre</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Si queda una demanda final negativa muy pequena, la conciliamos con regla trazable; si es material, se deja alerta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
           <t>El simulador</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Despues de tener L, cambiamos demanda final y calculamos impacto en produccion.</t>
         </is>
@@ -778,26 +791,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Mapa simple del proceso</t>
+          <t>Nombre de las matrices</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Lee de arriba hacia abajo. Cada paso tiene una hoja con un ejemplo.</t>
+          <t>Esta es la chuleta para leer el resto del Excel.</t>
         </is>
       </c>
     </row>
@@ -805,142 +819,405 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Paso</t>
+          <t>Nombre en archivo</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Nombre</t>
+          <t>Simbolo</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Formula</t>
+          <t>Nombre largo</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>En palabras</t>
+          <t>Que contiene</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Para que sirve</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n">
-        <v>1</v>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>V_oferta</t>
+        </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>COU</t>
+          <t>V</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Tabla de oferta V y utilizacion U.</t>
+          <t>Matriz de oferta/produccion</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Quien produce cada producto y quien lo compra.</t>
+          <t>Filas = sectores productores; columnas = productos.</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Sale del COU.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n">
-        <v>2</v>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>U_utilizacion</t>
+        </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Matriz de utilizacion intermedia</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Filas = productos; columnas = sectores compradores.</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Sale del COU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Y_demanda_final</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Matriz de demanda final</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Filas = productos; columnas = componentes de demanda final.</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Sale del COU depurado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>q_producto</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>q</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Vector de produccion por producto</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Suma de V por columna.</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Se usa para calcular D.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>D_market_share</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>D = V / q.</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Reparte un producto entre sectores productores.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Matriz de participaciones de mercado</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>D[i,p] = V[i,p] / q[p].</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Reparte productos entre sectores productores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Z_pre_conciliacion</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Z_pre</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Matriz insumo-producto previa</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>Z_pre = D @ U.</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Convierte producto x sector en sector x sector.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Cierre</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>RAS menor cuando aplica.</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Cierra negativos pequenos sin mover valor agregado residual.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>A y L</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>A = Z/g; L = (I-A)^-1.</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Prepara multiplicadores y simulador.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Choque</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Delta g = L @ Delta f.</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Calcula impacto de una variacion de demanda final.</t>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Primera MIP reconstruida antes del cierre menor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>ajuste_cierre</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>ajuste</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Tabla de conciliacion menor</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Compara demanda final antes/despues y ventas intermedias.</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Solo aparece si hubo cierre menor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Z_MIP / Z_final</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Matriz insumo-producto final</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Sector vendedor x sector comprador.</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Es la matriz publicada para el anio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>A_coef_tecnicos</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Matriz de coeficientes tecnicos</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>A[i,j] = Z[i,j] / g[j].</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Insumos requeridos por unidad de produccion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>B_ghosh_coef</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Matriz de coeficientes de Ghosh</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>B[i,j] = Z[i,j] / g[i].</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Distribucion de ventas del sector vendedor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>L_leontief</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Inversa de Leontief</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>L = (I - A)^-1.</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Base del simulador de choques de demanda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>G_ghosh_inversa</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Inversa de Ghosh</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>G = (I - B)^-1.</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Encadenamientos hacia adelante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>g_produccion</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Vector de produccion bruta</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Produccion total por sector.</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Escala A, B y los cierres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>f_demanda_final</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Vector de demanda final sectorial</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Demanda final transformada a sectores.</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>En simulador se modifica con shocks.</t>
         </is>
       </c>
     </row>
@@ -954,6 +1231,187 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Mapa simple del proceso</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Lee de arriba hacia abajo. Cada paso tiene una hoja con un ejemplo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Paso</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Nombre de matriz</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Formula</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>En palabras</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>V_oferta + U_utilizacion</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Matrices V y U.</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Quien produce cada producto y quien lo compra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>D_market_share</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>D = V / q.</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Reparte un producto entre sectores productores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Z_pre_conciliacion</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Z_pre = D @ U.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Convierte producto x sector en sector x sector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>ajuste_cierre + Z_MIP</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>RAS menor cuando aplica.</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Cierra negativos pequenos sin mover valor agregado residual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>A_coef_tecnicos + L_leontief</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>A = Z/g; L = (I-A)^-1.</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Prepara multiplicadores y simulador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>f_demanda_final + g_produccion</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Delta g = L @ Delta f.</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Calcula impacto de una variacion de demanda final.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -971,7 +1429,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Una celda de Z paso a paso</t>
+          <t>Matriz Z_pre: una celda paso a paso</t>
         </is>
       </c>
     </row>
@@ -1010,12 +1468,12 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Que queremos calcular</t>
+          <t>Matriz que queremos calcular</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Una celda de Z: cuanto vende el sector fila al sector columna.</t>
+          <t>Z_pre_conciliacion: una celda de la MIP antes del cierre menor.</t>
         </is>
       </c>
     </row>
@@ -1029,17 +1487,17 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>D: parte producida por Alimentos</t>
+          <t>Matriz D_market_share: parte producida por Alimentos</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>U: uso de Comercio</t>
+          <t>Matriz U_utilizacion: uso de Comercio</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Aporte D x U</t>
+          <t>Aporte a Z_pre = D x U</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1687,7 @@
     <row r="22">
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Z_pre calculada</t>
+          <t>Matriz Z_pre calculada</t>
         </is>
       </c>
       <c r="D22" s="4">
@@ -1240,7 +1698,7 @@
     <row r="23">
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Z_pre guardada por pipeline</t>
+          <t>Matriz Z_pre guardada por pipeline</t>
         </is>
       </c>
       <c r="D23" s="9" t="n">
@@ -1267,7 +1725,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Esta suma es una sola celda de la matriz Z previa. El pipeline repite esto para todos los pares sector-sector.</t>
+          <t>Esta suma es una sola celda de Z_pre_conciliacion. El pipeline repite esto para todos los pares sector-sector.</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1739,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1299,7 +1757,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>El cierre menor, sin drama</t>
+          <t>Matriz Z_MIP y ajuste_cierre</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1796,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Demanda final antes</t>
+          <t>f_demanda_final antes</t>
         </is>
       </c>
       <c r="B6" s="7" t="n">
@@ -1348,7 +1806,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Produccion bruta</t>
+          <t>g_produccion</t>
         </is>
       </c>
       <c r="B7" s="11" t="n">
@@ -1380,7 +1838,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Demanda final despues</t>
+          <t>f_demanda_final despues</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
@@ -1395,7 +1853,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>La produccion g y los totales de columna de Z.</t>
+          <t>g_produccion y los totales de columna de Z_pre.</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1879,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>No se cambia toda la matriz para que 'se vea bonita'. Se corrige un cierre pequeno, se deja la matriz previa y se registra el ajuste.</t>
+          <t>No se cambia toda la matriz sin registro. Se corrige un cierre pequeno, se deja Z_pre_conciliacion y se documenta ajuste_cierre.</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1893,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1453,7 +1911,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>De Z a coeficientes y multiplicadores</t>
+          <t>De Z_MIP a A_coef_tecnicos y L_leontief</t>
         </is>
       </c>
     </row>
@@ -1473,17 +1931,17 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Z_final hacia Comércio</t>
+          <t>Matriz Z_MIP hacia Comércio</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Produccion de Comércio</t>
+          <t>Vector g_produccion de Comércio</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>A = Z / g comprador</t>
+          <t>Matriz A_coef_tecnicos = Z / g comprador</t>
         </is>
       </c>
     </row>
@@ -1642,7 +2100,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Multiplicador simple mostrado</t>
+          <t>Multiplicador simple desde L_leontief</t>
         </is>
       </c>
       <c r="B18" s="9" t="n">
@@ -1664,7 +2122,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1691,7 +2149,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Simulador facil</t>
+          <t>Simulador facil con L_leontief</t>
         </is>
       </c>
     </row>
@@ -1706,7 +2164,7 @@
     <row r="4">
       <c r="I4" s="15" t="inlineStr">
         <is>
-          <t>L visible</t>
+          <t>Matriz L_leontief visible</t>
         </is>
       </c>
     </row>
@@ -1718,12 +2176,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>g_base</t>
+          <t>Vector g_base</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>f_base</t>
+          <t>Vector f_base</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1738,12 +2196,12 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Delta_g</t>
+          <t>Delta_g = L x Delta_f</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>g_nuevo</t>
+          <t>Vector g_nuevo</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -2069,13 +2527,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2112,79 +2570,79 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>COU</t>
+          <t>V_oferta / V</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Cuadro de oferta y utilizacion. Es la fuente antes de tener una MIP.</t>
+          <t>Oferta/produccion: que sector produce que producto.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>U_utilizacion / U</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Oferta/produccion: que sector produce que producto.</t>
+          <t>Utilizacion: que producto compra cada sector para producir.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>Y_demanda_final / Y</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Utilizacion: que producto compra cada sector para producir.</t>
+          <t>Demanda final: hogares, gobierno, inversion, exportaciones, etc.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>D_market_share / D</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Demanda final: hogares, gobierno, inversion, exportaciones, etc.</t>
+          <t>Matriz de reparto: de producto a sector productor.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Z_pre_conciliacion / Z_pre</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Matriz de reparto: de producto a sector productor.</t>
+          <t>Matriz insumo-producto antes del cierre menor.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Z</t>
+          <t>Z_MIP / Z</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Matriz insumo-producto: sector vendedor x sector comprador.</t>
+          <t>Matriz insumo-producto final: sector vendedor x sector comprador.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>A_coef_tecnicos / A</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -2196,7 +2654,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>L_leontief / L</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -2208,12 +2666,60 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>RAS</t>
+          <t>B_ghosh_coef / B</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Metodo de conciliacion para ajustar filas/columnas manteniendo restricciones.</t>
+          <t>Coeficientes de Ghosh para encadenamientos hacia adelante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>G_ghosh_inversa / G</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Inversa de Ghosh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>g_produccion / g</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Vector de produccion bruta por sector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>f_demanda_final / f</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Vector de demanda final por sector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>ajuste_cierre</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Tabla que documenta cierre menor cuando aplica.</t>
         </is>
       </c>
     </row>

</xml_diff>